<commit_message>
v0.1.0.0 — Büyük Kart Genişlemesi & Connected Core Sistemi
Connected Core (İç Yörünge) sistemi eklendi:
- Vector: 7 Connected Core (index 178-184)
- Leila: 7 Connected Core (index 185-191) + ElementalShield çoklu animasyon
- Cyclone: 6 Connected Core (index 192-197) + CircuitOverload sayaç animasyonu

Yeni kartlar:
- Vector: WormHole + Siege Rain Calamity (index 198-199)
- Leila: 12 kart — Individuality/Calamity/Utility (index 200-211)
- Cyclone: 12 kart — Identity/Calamity/Individuality/Utility (index 212-223)

Yeni Core tipleri: Tracer Core (iz efekti), Spike Core, Leech Nova Core
Yeni Calamity: Deep Freeze, Wildfire, Glitch Bomb, System Crash, Antivirus Rain, Decay Field
Momentum Burst emoji düzeltmesi (⚡ çakışması giderildi → 💨)
Excel kart dosyaları güncellendi, güncelleme notları ve todolist güncellendi

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cycloneCards.xlsx
+++ b/cycloneCards.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,10 @@
       <b val="1"/>
       <color rgb="00FFAA00"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -127,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -170,6 +174,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -536,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1897,6 +1904,492 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>Glitch Pulse Core</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>Every 4s: applies Glitch to 1 random enemy within 80px</t>
+        </is>
+      </c>
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>Her 4s: 80px icerisinde 1 rastgele dusmana Glitch uygular</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>Nadiren Gorulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>Shadow Core</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>After dash: for 3s orbit speeds up and deals 1 dmg/s to enemies within 50px</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>Dash sonrasi 3s: orbit hizlanir ve 50px cevresine 1 hasar/s uygular</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>Data Drain Core</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>If a Glitched enemy is within 60px: gain +1 HP per second</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>Glitchli dusman 60px icindeyse her saniye +1 HP kazanilir</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>Nadiren Gorulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>Virus Beacon Core</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>When an Antivirused enemy dies within 80px: for 3s spreads 1 stack to enemies in 100px</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>Antiviruslu dusman 80px icinde olurse 3s boyunca 100px cevresine 1 stack yayar</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>Rogue's Eye Core</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>Every 7s: marks nearest enemy for 3s (marked enemies take 10%% more damage)</t>
+        </is>
+      </c>
+      <c r="D58" s="15" t="inlineStr">
+        <is>
+          <t>Her 7s: en yakin dusmani 3s isaretler (isaretli dusman %%10 fazla hasar alir)</t>
+        </is>
+      </c>
+      <c r="E58" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>Circuit Overload Core</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>When Circuit Breaker triggers: for 3s continuously Glitches enemies within 90px. Animation shows CB counter progress.</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>Circuit Breaker tetiklenince 3s boyunca 90px cevresine surekli Glitch uygular. Animasyon sayac ilerlemesini gosterir.</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>Destansı</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>Tracer Core</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>On hit: leaves a 1s trail; enemies crossing the trail get 0.5s slow</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>Vuruşta 1s iz bırakır; izden geçen düşman 0.5s yavaşlar</t>
+        </is>
+      </c>
+      <c r="E60" s="15" t="inlineStr">
+        <is>
+          <t>Nadiren Gorulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>Spike Core</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>On hit: if target has 3 Decay stacks, instantly triggers Decay death burst</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>3 Decay stack varsa: anında Decay patlaması tetiklenir</t>
+        </is>
+      </c>
+      <c r="E61" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>Leech Nova Core</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>Kimlik</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>On kill: +2 HP, Glitch enemies within 80px for 1s</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>Öldürünce: +2 HP, 80px çevresine 1s Glitch</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr">
+        <is>
+          <t>Destansı</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>Glitch Bomb</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>Felaket</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>Glitches all enemies within 120px of target for 4s</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>Seçilen 120px alana 4s Glitch uygular</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>System Crash</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>Felaket</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>All Glitched enemies in the Yard lose 30%% of their current HP</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>Tüm Glitch'li düşmanlar mevcut HP'nin %%30'unu kaybeder</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>Destansı</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>Antivirus Rain</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Felaket</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>For 3s: every 0.5s, applies 1 Antivirus stack to all enemies</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>3s boyunca her 0.5s: tüm düşmanlara 1 Antivirus stack</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>Decay Field</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>Felaket</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>5s: aura on selected 100px area; enemies inside get 1 Decay stack per second</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>5s: 100px alana aura; giren düşmanlar her 1s'de 1 Decay alır</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>Destansı</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>Decay Harvest</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>Bireysellik</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>Whenever a Decay death burst triggers: +2 HP</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>Decay patlaması tetiklenince: +2 HP</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="inlineStr">
+        <is>
+          <t>Nadiren Gorulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>Ghost Step</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>Bireysellik</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>After dash: 1.5s damage immunity (5s cooldown)</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>Dash sonrası 1.5s hasar bağışıklığı (5s bekleme süresi)</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>Overclock Protocol</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Bireysellik</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Circuit Breaker counter builds 2x faster</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Circuit Breaker sayacı 2x hızlı dolar</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>Destansı</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>Decay Amp</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>Yardimci</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>Decay death burst damage per stack: 2 -&gt; 3</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>Decay patlaması hasarı: stack başına 2 -&gt; 3</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>Nadiren Gorulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>Static Link</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Yardimci</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>Static Core: if target is Glitched, slow duration is 2x longer</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>Static Core: hedef Glitch'liyse slow süresi 2x uzar</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>

</xml_diff>